<commit_message>
(TEDSWS-559 - Mapping sdk1.15 to ePO_4.0.0): Add columns for sdk1.14 and sdk1.15 to all conceptual mapping files
</commit_message>
<xml_diff>
--- a/mappings/package_eforms_sdk1.15_epo4.0/transformation/conceptual_mappings.xlsx
+++ b/mappings/package_eforms_sdk1.15_epo4.0/transformation/conceptual_mappings.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" state="visible" r:id="rId3"/>
@@ -68,7 +68,7 @@
     <t xml:space="preserve">Mapping Version</t>
   </si>
   <si>
-    <t xml:space="preserve">1.1.0</t>
+    <t xml:space="preserve">1.2.1</t>
   </si>
   <si>
     <t xml:space="preserve">Version of the Mapping Suite (use semantic versioning, see https://semver.org/ )</t>

</xml_diff>